<commit_message>
feat: etude complete neurones caches 6-6-1 a 6-30-1
- 25 architectures testees, 10 repetitions chacune (250 entrainements)
- Meilleure architecture : 6-8-1 (MSE=0.549)
- Tendance : MSE augmente pour H > 13 (surapprentissage)
- Graphique publication-quality mis a jour
</commit_message>
<xml_diff>
--- a/results/architecture_search/hidden_neurons_results.xlsx
+++ b/results/architecture_search/hidden_neurons_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,6 +608,586 @@
         <v>0.0359083779</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.5826133125</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.7629742604999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6213512092</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.1341099417</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.03344861</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.021990687</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0132594748</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.0651107695</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.5796475575</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.7610825907</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.6198810331</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.1283368292</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0304724633</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0200211783</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0159661719</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0593174286</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.5748405022999999</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.7579650726</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.6108942356</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.1189794579</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.0278178227</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0181507853</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.0162392277</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.0541499287</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.5831154575</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.7633675109</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.6097437487</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.1350874127</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0297534235</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.019634172</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.0121222083</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0579177522</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.5836523732</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7636868322</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.6141046046</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.136132568</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.031819454</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0208517514</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.0148526108</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0619394688</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5844674918</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.7641984606</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.6205311335</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.1377192708</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0329434613</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0216380348</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.0189551913</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0641274515</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5970046443</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.7721740802</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.6189111949</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.1621239815</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.0424506865</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0274195939</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.0181008001</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0826341323</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.6035829637</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.7767652529</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.6190358476</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.17492928</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.0227843036</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0147886968</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.0082709185</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.0443517248</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.5954691188</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.7713605023</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.6155310761</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.159134941</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0333563329</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0217277309</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0137268196</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.0649311437</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5968644895</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.772331557</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.6186734581</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.1618511573</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.0298592342</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0191951974</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.0124341766</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.0581237222</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.6033935329</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.7766150232</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.6167275494</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.1745605357</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.0253034226</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0162061298</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.013033552</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.0492554195</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.5974203423</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.7728728429</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.616282369</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.1629331755</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0144779231</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0093760878</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.0076867295</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.0281825976</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>23</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.6109259505</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.7814325809</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.6222893126</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.1892230734</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0266375006</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0170021181</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.0099445127</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.051852324</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>24</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.6107673447999999</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.7814112347</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.6217367023</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.1889143329</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0201154355</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.0127994918</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.0105746535</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.0391565295</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>25</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.6052980474</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.7778013964</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.6239790633</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.1782678467</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0278013531</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0179731789</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.0140683621</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.0541178691</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>26</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.6031673027</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.7765737712</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.6191303419</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.174120158</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0155187527</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.010023999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.009371091999999999</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.0302086674</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>27</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.6173843682</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.7855424686</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.6216392492</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.2017949725</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0274886899</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.017532777</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.0108749455</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.0535092416</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>28</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.6124956302</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.7825126495</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.6237399501000001</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1.1922785981</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0203517305</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.0130224257</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.0113576763</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.0396164992</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>29</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.6285474256</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.7927680083999999</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.6264739904</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.2235248816</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.0129110714</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.0081431174</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.0060572743</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.0251325778</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>30</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.6217772648</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.78846299</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.6268887391</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.2103461462</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.015949611</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.0101675026</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.0086271144</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.0310473723</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: etude neurones caches 6-6-1 a 6-15-1 (10 architectures)
- Range reduit de 25 a 10 architectures
- Meilleure architecture : 6-8-1 (MSE=0.549)
</commit_message>
<xml_diff>
--- a/results/architecture_search/hidden_neurons_results.xlsx
+++ b/results/architecture_search/hidden_neurons_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -753,441 +753,6 @@
         <v>0.0619394688</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>16</v>
-      </c>
-      <c r="B12" t="n">
-        <v>0.5844674918</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.7641984606</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.6205311335</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1.1377192708</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.0329434613</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.0216380348</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.0189551913</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.0641274515</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>17</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0.5970046443</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.7721740802</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.6189111949</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1.1621239815</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.0424506865</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.0274195939</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.0181008001</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.0826341323</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>18</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0.6035829637</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.7767652529</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.6190358476</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1.17492928</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.0227843036</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.0147886968</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.0082709185</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.0443517248</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>19</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.5954691188</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.7713605023</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.6155310761</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.159134941</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.0333563329</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.0217277309</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.0137268196</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.0649311437</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>20</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0.5968644895</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.772331557</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.6186734581</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1.1618511573</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.0298592342</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.0191951974</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.0124341766</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0.0581237222</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>21</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.6033935329</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.7766150232</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.6167275494</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1.1745605357</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.0253034226</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.0162061298</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.013033552</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.0492554195</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>22</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.5974203423</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.7728728429</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.616282369</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1.1629331755</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.0144779231</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.0093760878</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.0076867295</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.0281825976</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>23</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.6109259505</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.7814325809</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.6222893126</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1.1892230734</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.0266375006</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.0170021181</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.0099445127</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.051852324</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>24</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.6107673447999999</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.7814112347</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.6217367023</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1.1889143329</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.0201154355</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.0127994918</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.0105746535</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.0391565295</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>25</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.6052980474</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.7778013964</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.6239790633</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1.1782678467</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.0278013531</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.0179731789</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.0140683621</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.0541178691</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>26</v>
-      </c>
-      <c r="B22" t="n">
-        <v>0.6031673027</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.7765737712</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.6191303419</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1.174120158</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.0155187527</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.010023999</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.009371091999999999</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.0302086674</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>27</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.6173843682</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.7855424686</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.6216392492</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1.2017949725</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.0274886899</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.017532777</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.0108749455</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.0535092416</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>28</v>
-      </c>
-      <c r="B24" t="n">
-        <v>0.6124956302</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.7825126495</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.6237399501000001</v>
-      </c>
-      <c r="E24" t="n">
-        <v>1.1922785981</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.0203517305</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.0130224257</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.0113576763</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0.0396164992</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>29</v>
-      </c>
-      <c r="B25" t="n">
-        <v>0.6285474256</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.7927680083999999</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.6264739904</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1.2235248816</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.0129110714</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.0081431174</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.0060572743</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0.0251325778</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>30</v>
-      </c>
-      <c r="B26" t="n">
-        <v>0.6217772648</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.78846299</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.6268887391</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1.2103461462</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.015949611</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.0101675026</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.0086271144</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0.0310473723</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: mise a jour Excel avec 8 decimales
</commit_message>
<xml_diff>
--- a/results/architecture_search/hidden_neurons_results.xlsx
+++ b/results/architecture_search/hidden_neurons_results.xlsx
@@ -468,28 +468,28 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5536795382</v>
+        <v>0.55367954</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7435831171</v>
+        <v>0.74358312</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6142097114</v>
+        <v>0.61420971</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0777877117</v>
+        <v>1.07778771</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0406292223</v>
+        <v>0.04062922</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0276348739</v>
+        <v>0.02763487</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0185249396</v>
+        <v>0.01852494</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0790884862</v>
+        <v>0.07908849</v>
       </c>
     </row>
     <row r="3">
@@ -497,28 +497,28 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.5828314613</v>
+        <v>0.58283146</v>
       </c>
       <c r="C3" t="n">
-        <v>0.762558125</v>
+        <v>0.76255812</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6224097703</v>
+        <v>0.62240977</v>
       </c>
       <c r="E3" t="n">
-        <v>1.1345345882</v>
+        <v>1.13453459</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0558915631</v>
+        <v>0.05589156</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0365590924</v>
+        <v>0.03655909</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0276880438</v>
+        <v>0.02768804</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1087980243</v>
+        <v>0.10879802</v>
       </c>
     </row>
     <row r="4">
@@ -526,28 +526,28 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.5488925222</v>
+        <v>0.54889252</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7405019313</v>
+        <v>0.74050193</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6028052404000001</v>
+        <v>0.60280524</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0684693483</v>
+        <v>1.06846935</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0345013223</v>
+        <v>0.03450132</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0234395379</v>
+        <v>0.02343954</v>
       </c>
       <c r="H4" t="n">
-        <v>0.017958943</v>
+        <v>0.01795894</v>
       </c>
       <c r="I4" t="n">
-        <v>0.06715997009999999</v>
+        <v>0.06715997</v>
       </c>
     </row>
     <row r="5">
@@ -555,28 +555,28 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.582285367</v>
+        <v>0.58228537</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7627600325</v>
+        <v>0.76276003</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6276085923</v>
+        <v>0.62760859</v>
       </c>
       <c r="E5" t="n">
-        <v>1.1334715659</v>
+        <v>1.13347157</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0341648523</v>
+        <v>0.03416485</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0219658775</v>
+        <v>0.02196588</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0214693397</v>
+        <v>0.02146934</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0665050006</v>
+        <v>0.06650499999999999</v>
       </c>
     </row>
     <row r="6">
@@ -584,28 +584,28 @@
         <v>10</v>
       </c>
       <c r="B6" t="n">
-        <v>0.5549944483</v>
+        <v>0.55499445</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7448771874</v>
+        <v>0.74487719</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6097403201</v>
+        <v>0.60974032</v>
       </c>
       <c r="E6" t="n">
-        <v>1.0803473039</v>
+        <v>1.0803473</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0184467997</v>
+        <v>0.0184468</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0123460071</v>
+        <v>0.01234601</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0080641663</v>
+        <v>0.008064170000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0359083779</v>
+        <v>0.03590838</v>
       </c>
     </row>
     <row r="7">
@@ -613,28 +613,28 @@
         <v>11</v>
       </c>
       <c r="B7" t="n">
-        <v>0.5826133125</v>
+        <v>0.5826133100000001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7629742604999999</v>
+        <v>0.76297426</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6213512092</v>
+        <v>0.62135121</v>
       </c>
       <c r="E7" t="n">
-        <v>1.1341099417</v>
+        <v>1.13410994</v>
       </c>
       <c r="F7" t="n">
         <v>0.03344861</v>
       </c>
       <c r="G7" t="n">
-        <v>0.021990687</v>
+        <v>0.02199069</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0132594748</v>
+        <v>0.01325947</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0651107695</v>
+        <v>0.06511077</v>
       </c>
     </row>
     <row r="8">
@@ -642,28 +642,28 @@
         <v>12</v>
       </c>
       <c r="B8" t="n">
-        <v>0.5796475575</v>
+        <v>0.57964756</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7610825907</v>
+        <v>0.76108259</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6198810331</v>
+        <v>0.6198810300000001</v>
       </c>
       <c r="E8" t="n">
-        <v>1.1283368292</v>
+        <v>1.12833683</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0304724633</v>
+        <v>0.03047246</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0200211783</v>
+        <v>0.02002118</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0159661719</v>
+        <v>0.01596617</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0593174286</v>
+        <v>0.05931743</v>
       </c>
     </row>
     <row r="9">
@@ -671,28 +671,28 @@
         <v>13</v>
       </c>
       <c r="B9" t="n">
-        <v>0.5748405022999999</v>
+        <v>0.5748405</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7579650726</v>
+        <v>0.75796507</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6108942356</v>
+        <v>0.61089424</v>
       </c>
       <c r="E9" t="n">
-        <v>1.1189794579</v>
+        <v>1.11897946</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0278178227</v>
+        <v>0.02781782</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0181507853</v>
+        <v>0.01815079</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0162392277</v>
+        <v>0.01623923</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0541499287</v>
+        <v>0.05414993</v>
       </c>
     </row>
     <row r="10">
@@ -700,28 +700,28 @@
         <v>14</v>
       </c>
       <c r="B10" t="n">
-        <v>0.5831154575</v>
+        <v>0.58311546</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7633675109</v>
+        <v>0.76336751</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6097437487</v>
+        <v>0.60974375</v>
       </c>
       <c r="E10" t="n">
-        <v>1.1350874127</v>
+        <v>1.13508741</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0297534235</v>
+        <v>0.02975342</v>
       </c>
       <c r="G10" t="n">
-        <v>0.019634172</v>
+        <v>0.01963417</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0121222083</v>
+        <v>0.01212221</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0579177522</v>
+        <v>0.05791775</v>
       </c>
     </row>
     <row r="11">
@@ -729,28 +729,28 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>0.5836523732</v>
+        <v>0.58365237</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7636868322</v>
+        <v>0.76368683</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6141046046</v>
+        <v>0.6141046</v>
       </c>
       <c r="E11" t="n">
-        <v>1.136132568</v>
+        <v>1.13613257</v>
       </c>
       <c r="F11" t="n">
-        <v>0.031819454</v>
+        <v>0.03181945</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0208517514</v>
+        <v>0.02085175</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0148526108</v>
+        <v>0.01485261</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0619394688</v>
+        <v>0.06193947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>